<commit_message>
ANS-006-168 - Mise à jour du séjour  (#428)
* update séjour

* enrichissement sejour

* maj séjour

* fix

* update

* suppression jdv

* suppression modaliteentree et sortie

* update

* update PR

* update sushi-config 26fba3e241bfd5c7122250660217b619eef2f39f
</commit_message>
<xml_diff>
--- a/441-rc---tdduipatient-birthdate/ig/CodeSystem-tddui-discriminator.xlsx
+++ b/441-rc---tdduipatient-birthdate/ig/CodeSystem-tddui-discriminator.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-26T15:34:05+00:00</t>
+    <t>2026-02-26T16:28:52+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -78,7 +78,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>FRANCE</t>
+    <t>France</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>